<commit_message>
Added achievement table below each game and added basic sort by features.
</commit_message>
<xml_diff>
--- a/Steam_Games.xlsx
+++ b/Steam_Games.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CJ\Documents\My Projects\My Skill Development\game-achievement-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EB33888-36C5-47AD-949D-DD3709D607F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE1AFFC6-F2B1-419C-B62E-75849A810B9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="13284" windowHeight="13416" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>ID</t>
   </si>
@@ -84,6 +84,9 @@
   </si>
   <si>
     <t>Cuphead</t>
+  </si>
+  <si>
+    <t>release_year</t>
   </si>
 </sst>
 </file>
@@ -119,9 +122,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -144,9 +146,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{507F0839-0555-426B-B7DB-068B4BAF2678}" name="Table1" displayName="Table1" ref="A1:D13" totalsRowShown="0">
-  <autoFilter ref="A1:D13" xr:uid="{507F0839-0555-426B-B7DB-068B4BAF2678}"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{507F0839-0555-426B-B7DB-068B4BAF2678}" name="Table1" displayName="Table1" ref="A1:E13" totalsRowShown="0">
+  <autoFilter ref="A1:E13" xr:uid="{507F0839-0555-426B-B7DB-068B4BAF2678}"/>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{3E161485-89FB-41E6-A63E-4664D0B0ECB0}" name="ID">
       <calculatedColumnFormula>ROW()-1</calculatedColumnFormula>
     </tableColumn>
@@ -155,6 +157,7 @@
     <tableColumn id="4" xr3:uid="{A71223AC-FD24-4499-A224-DD876F6C628B}" name="game_link" dataDxfId="0">
       <calculatedColumnFormula>"https://steamdb.info/app/"&amp;Table1[[#This Row],[game_id]]&amp;"/stats/"</calculatedColumnFormula>
     </tableColumn>
+    <tableColumn id="5" xr3:uid="{668B1B8A-AE89-4A14-89D0-E329F1EAD30A}" name="release_year"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -423,10 +426,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -439,8 +442,11 @@
       <c r="D1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <f t="shared" ref="A2:A12" si="0">ROW()-1</f>
         <v>1</v>
@@ -455,8 +461,11 @@
         <f>"https://steamdb.info/app/"&amp;Table1[[#This Row],[game_id]]&amp;"/stats/"</f>
         <v>https://steamdb.info/app/2358720/stats/</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E2">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -471,8 +480,11 @@
         <f>"https://steamdb.info/app/"&amp;Table1[[#This Row],[game_id]]&amp;"/stats/"</f>
         <v>https://steamdb.info/app/1627720/stats/</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E3">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -487,8 +499,11 @@
         <f>"https://steamdb.info/app/"&amp;Table1[[#This Row],[game_id]]&amp;"/stats/"</f>
         <v>https://steamdb.info/app/1245620/stats/</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E4">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -503,8 +518,11 @@
         <f>"https://steamdb.info/app/"&amp;Table1[[#This Row],[game_id]]&amp;"/stats/"</f>
         <v>https://steamdb.info/app/814380/stats/</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E5">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -519,8 +537,11 @@
         <f>"https://steamdb.info/app/"&amp;Table1[[#This Row],[game_id]]&amp;"/stats/"</f>
         <v>https://steamdb.info/app/2622380/stats/</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E6">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -535,8 +556,11 @@
         <f>"https://steamdb.info/app/"&amp;Table1[[#This Row],[game_id]]&amp;"/stats/"</f>
         <v>https://steamdb.info/app/1030300/stats/</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E7">
+        <v>2017</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -551,8 +575,11 @@
         <f>"https://steamdb.info/app/"&amp;Table1[[#This Row],[game_id]]&amp;"/stats/"</f>
         <v>https://steamdb.info/app/367520/stats/</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E8">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -567,8 +594,11 @@
         <f>"https://steamdb.info/app/"&amp;Table1[[#This Row],[game_id]]&amp;"/stats/"</f>
         <v>https://steamdb.info/app/2138710/stats/</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E9">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -583,8 +613,11 @@
         <f>"https://steamdb.info/app/"&amp;Table1[[#This Row],[game_id]]&amp;"/stats/"</f>
         <v>https://steamdb.info/app/1145360/stats/</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E10">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -599,8 +632,11 @@
         <f>"https://steamdb.info/app/"&amp;Table1[[#This Row],[game_id]]&amp;"/stats/"</f>
         <v>https://steamdb.info/app/1145350/stats/</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E11">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -615,8 +651,11 @@
         <f>"https://steamdb.info/app/"&amp;Table1[[#This Row],[game_id]]&amp;"/stats/"</f>
         <v>https://steamdb.info/app/1903340/stats/</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E12">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13">
         <f>ROW()-1</f>
         <v>12</v>
@@ -627,9 +666,12 @@
       <c r="C13">
         <v>268910</v>
       </c>
-      <c r="D13" s="1" t="str">
+      <c r="D13" t="str">
         <f>"https://steamdb.info/app/"&amp;Table1[[#This Row],[game_id]]&amp;"/stats/"</f>
         <v>https://steamdb.info/app/268910/stats/</v>
+      </c>
+      <c r="E13">
+        <v>2017</v>
       </c>
     </row>
   </sheetData>

</xml_diff>